<commit_message>
feat: Add detailed LEAN cocotte workshop scenario and all associated supporting materials.
</commit_message>
<xml_diff>
--- a/OI/A2 TRS/TP analyse centre usinage.xlsx
+++ b/OI/A2 TRS/TP analyse centre usinage.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cfaicentre-my.sharepoint.com/personal/s_jaubert_poleformation-uimmcvdl_fr/Documents/Bachelor/2026 BACH/Stage 2 TRS/TRS/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cfaicentre-my.sharepoint.com/personal/s_jaubert_poleformation-uimmcvdl_fr/Documents/00FC/OI/A2 TRS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="43" documentId="13_ncr:1_{FBACCD43-1F08-4960-A2F5-622601195D11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8F2B3651-C245-4497-AC38-D744216D8C94}"/>
+  <xr:revisionPtr revIDLastSave="44" documentId="13_ncr:1_{FBACCD43-1F08-4960-A2F5-622601195D11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3CF7664F-A2D2-4A6C-AF5E-ADCAB5E0AD38}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{0B317174-6610-4FA1-8F85-0AE134DA76FE}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0B317174-6610-4FA1-8F85-0AE134DA76FE}"/>
   </bookViews>
   <sheets>
     <sheet name="TRS" sheetId="1" r:id="rId1"/>
@@ -268,9 +268,6 @@
     <t>Coûts de défaillance</t>
   </si>
   <si>
-    <t>Travail à faire : Voir les deux onglets - Rendre par mail ou déposer sur le serveur ce fichier Excel</t>
-  </si>
-  <si>
     <t>coût de défaillance et en mettant en évidence les sous-systèmes responsables de 80% des coûts</t>
   </si>
   <si>
@@ -317,6 +314,9 @@
   </si>
   <si>
     <t>Le centre C31 a une cadence de</t>
+  </si>
+  <si>
+    <t>Travail à faire : Voir les deux onglets</t>
   </si>
 </sst>
 </file>
@@ -483,11 +483,27 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -498,22 +514,6 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -839,39 +839,39 @@
       <c r="A1" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="B1" s="19"/>
-      <c r="C1" s="19"/>
-      <c r="D1" s="19"/>
-      <c r="E1" s="19"/>
-      <c r="F1" s="19"/>
-      <c r="G1" s="19"/>
-      <c r="H1" s="19"/>
+      <c r="B1" s="23"/>
+      <c r="C1" s="23"/>
+      <c r="D1" s="23"/>
+      <c r="E1" s="23"/>
+      <c r="F1" s="23"/>
+      <c r="G1" s="23"/>
+      <c r="H1" s="23"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A3" s="20" t="s">
-        <v>77</v>
-      </c>
-      <c r="B3" s="20"/>
-      <c r="C3" s="20"/>
-      <c r="D3" s="20"/>
-      <c r="E3" s="20"/>
-      <c r="F3" s="20"/>
-      <c r="G3" s="20"/>
-      <c r="H3" s="20"/>
-      <c r="I3" s="20"/>
-      <c r="J3" s="20"/>
+      <c r="A3" s="24" t="s">
+        <v>93</v>
+      </c>
+      <c r="B3" s="24"/>
+      <c r="C3" s="24"/>
+      <c r="D3" s="24"/>
+      <c r="E3" s="24"/>
+      <c r="F3" s="24"/>
+      <c r="G3" s="24"/>
+      <c r="H3" s="24"/>
+      <c r="I3" s="24"/>
+      <c r="J3" s="24"/>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A4" s="20"/>
-      <c r="B4" s="20"/>
-      <c r="C4" s="20"/>
-      <c r="D4" s="20"/>
-      <c r="E4" s="20"/>
-      <c r="F4" s="20"/>
-      <c r="G4" s="20"/>
-      <c r="H4" s="20"/>
-      <c r="I4" s="20"/>
-      <c r="J4" s="20"/>
+      <c r="A4" s="24"/>
+      <c r="B4" s="24"/>
+      <c r="C4" s="24"/>
+      <c r="D4" s="24"/>
+      <c r="E4" s="24"/>
+      <c r="F4" s="24"/>
+      <c r="G4" s="24"/>
+      <c r="H4" s="24"/>
+      <c r="I4" s="24"/>
+      <c r="J4" s="24"/>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
@@ -890,7 +890,7 @@
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
@@ -905,39 +905,39 @@
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B16" s="26" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C16" s="26"/>
       <c r="D16" s="26"/>
       <c r="E16" s="26"/>
       <c r="F16" s="26"/>
       <c r="G16" s="26"/>
-      <c r="H16" s="25">
+      <c r="H16" s="19">
         <v>15.7</v>
       </c>
       <c r="I16" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="17" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="B17" s="25" t="s">
         <v>91</v>
       </c>
-    </row>
-    <row r="17" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="B17" s="24" t="s">
-        <v>92</v>
-      </c>
-      <c r="C17" s="24"/>
-      <c r="D17" s="24"/>
-      <c r="E17" s="24"/>
-      <c r="F17" s="24"/>
-      <c r="G17" s="24"/>
-      <c r="H17" s="25">
+      <c r="C17" s="25"/>
+      <c r="D17" s="25"/>
+      <c r="E17" s="25"/>
+      <c r="F17" s="25"/>
+      <c r="G17" s="25"/>
+      <c r="H17" s="19">
         <v>14.4</v>
       </c>
       <c r="I17" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="18" spans="1:23" x14ac:dyDescent="0.25">
@@ -958,7 +958,7 @@
     </row>
     <row r="22" spans="1:23" x14ac:dyDescent="0.25">
       <c r="B22" s="9" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="23" spans="1:23" x14ac:dyDescent="0.25">
@@ -968,17 +968,17 @@
     </row>
     <row r="24" spans="1:23" x14ac:dyDescent="0.25">
       <c r="B24" s="9" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="25" spans="1:23" x14ac:dyDescent="0.25">
       <c r="B25" s="9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="26" spans="1:23" x14ac:dyDescent="0.25">
       <c r="B26" s="9" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="28" spans="1:23" x14ac:dyDescent="0.25">
@@ -1123,7 +1123,7 @@
     </row>
     <row r="30" spans="1:23" s="1" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="4" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B30" s="6">
         <v>3</v>
@@ -1193,58 +1193,58 @@
       </c>
     </row>
     <row r="31" spans="1:23" s="1" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="27" t="s">
-        <v>82</v>
-      </c>
-      <c r="B31" s="28"/>
-      <c r="C31" s="28"/>
-      <c r="D31" s="28"/>
-      <c r="E31" s="28"/>
-      <c r="F31" s="28"/>
-      <c r="G31" s="28"/>
-      <c r="H31" s="28"/>
-      <c r="I31" s="28"/>
-      <c r="J31" s="28"/>
-      <c r="K31" s="28"/>
-      <c r="L31" s="28"/>
-      <c r="M31" s="28"/>
-      <c r="N31" s="28"/>
-      <c r="O31" s="28"/>
-      <c r="P31" s="28"/>
-      <c r="Q31" s="28"/>
-      <c r="R31" s="28"/>
-      <c r="S31" s="28"/>
-      <c r="T31" s="28"/>
-      <c r="U31" s="28"/>
-      <c r="V31" s="28"/>
-      <c r="W31" s="28"/>
+      <c r="A31" s="20" t="s">
+        <v>81</v>
+      </c>
+      <c r="B31" s="21"/>
+      <c r="C31" s="21"/>
+      <c r="D31" s="21"/>
+      <c r="E31" s="21"/>
+      <c r="F31" s="21"/>
+      <c r="G31" s="21"/>
+      <c r="H31" s="21"/>
+      <c r="I31" s="21"/>
+      <c r="J31" s="21"/>
+      <c r="K31" s="21"/>
+      <c r="L31" s="21"/>
+      <c r="M31" s="21"/>
+      <c r="N31" s="21"/>
+      <c r="O31" s="21"/>
+      <c r="P31" s="21"/>
+      <c r="Q31" s="21"/>
+      <c r="R31" s="21"/>
+      <c r="S31" s="21"/>
+      <c r="T31" s="21"/>
+      <c r="U31" s="21"/>
+      <c r="V31" s="21"/>
+      <c r="W31" s="21"/>
     </row>
     <row r="32" spans="1:23" s="1" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="27" t="s">
+      <c r="A32" s="20" t="s">
         <v>3</v>
       </c>
-      <c r="B32" s="28"/>
-      <c r="C32" s="28"/>
-      <c r="D32" s="28"/>
-      <c r="E32" s="28"/>
-      <c r="F32" s="28"/>
-      <c r="G32" s="28"/>
-      <c r="H32" s="28"/>
-      <c r="I32" s="28"/>
-      <c r="J32" s="28"/>
-      <c r="K32" s="28"/>
-      <c r="L32" s="28"/>
-      <c r="M32" s="28"/>
-      <c r="N32" s="28"/>
-      <c r="O32" s="28"/>
-      <c r="P32" s="28"/>
-      <c r="Q32" s="28"/>
-      <c r="R32" s="28"/>
-      <c r="S32" s="28"/>
-      <c r="T32" s="28"/>
-      <c r="U32" s="28"/>
-      <c r="V32" s="28"/>
-      <c r="W32" s="28"/>
+      <c r="B32" s="21"/>
+      <c r="C32" s="21"/>
+      <c r="D32" s="21"/>
+      <c r="E32" s="21"/>
+      <c r="F32" s="21"/>
+      <c r="G32" s="21"/>
+      <c r="H32" s="21"/>
+      <c r="I32" s="21"/>
+      <c r="J32" s="21"/>
+      <c r="K32" s="21"/>
+      <c r="L32" s="21"/>
+      <c r="M32" s="21"/>
+      <c r="N32" s="21"/>
+      <c r="O32" s="21"/>
+      <c r="P32" s="21"/>
+      <c r="Q32" s="21"/>
+      <c r="R32" s="21"/>
+      <c r="S32" s="21"/>
+      <c r="T32" s="21"/>
+      <c r="U32" s="21"/>
+      <c r="V32" s="21"/>
+      <c r="W32" s="21"/>
     </row>
     <row r="33" spans="1:23" s="1" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="4" t="s">
@@ -1389,31 +1389,31 @@
       </c>
     </row>
     <row r="35" spans="1:23" s="1" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="27" t="s">
+      <c r="A35" s="20" t="s">
         <v>2</v>
       </c>
-      <c r="B35" s="28"/>
-      <c r="C35" s="28"/>
-      <c r="D35" s="28"/>
-      <c r="E35" s="28"/>
-      <c r="F35" s="28"/>
-      <c r="G35" s="28"/>
-      <c r="H35" s="28"/>
-      <c r="I35" s="28"/>
-      <c r="J35" s="28"/>
-      <c r="K35" s="28"/>
-      <c r="L35" s="28"/>
-      <c r="M35" s="28"/>
-      <c r="N35" s="28"/>
-      <c r="O35" s="28"/>
-      <c r="P35" s="28"/>
-      <c r="Q35" s="28"/>
-      <c r="R35" s="28"/>
-      <c r="S35" s="28"/>
-      <c r="T35" s="28"/>
-      <c r="U35" s="28"/>
-      <c r="V35" s="28"/>
-      <c r="W35" s="28"/>
+      <c r="B35" s="21"/>
+      <c r="C35" s="21"/>
+      <c r="D35" s="21"/>
+      <c r="E35" s="21"/>
+      <c r="F35" s="21"/>
+      <c r="G35" s="21"/>
+      <c r="H35" s="21"/>
+      <c r="I35" s="21"/>
+      <c r="J35" s="21"/>
+      <c r="K35" s="21"/>
+      <c r="L35" s="21"/>
+      <c r="M35" s="21"/>
+      <c r="N35" s="21"/>
+      <c r="O35" s="21"/>
+      <c r="P35" s="21"/>
+      <c r="Q35" s="21"/>
+      <c r="R35" s="21"/>
+      <c r="S35" s="21"/>
+      <c r="T35" s="21"/>
+      <c r="U35" s="21"/>
+      <c r="V35" s="21"/>
+      <c r="W35" s="21"/>
     </row>
     <row r="36" spans="1:23" s="1" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="4" t="s">
@@ -1558,31 +1558,31 @@
       </c>
     </row>
     <row r="38" spans="1:23" s="1" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="27" t="s">
+      <c r="A38" s="20" t="s">
         <v>7</v>
       </c>
-      <c r="B38" s="28"/>
-      <c r="C38" s="28"/>
-      <c r="D38" s="28"/>
-      <c r="E38" s="28"/>
-      <c r="F38" s="28"/>
-      <c r="G38" s="28"/>
-      <c r="H38" s="28"/>
-      <c r="I38" s="28"/>
-      <c r="J38" s="28"/>
-      <c r="K38" s="28"/>
-      <c r="L38" s="28"/>
-      <c r="M38" s="28"/>
-      <c r="N38" s="28"/>
-      <c r="O38" s="28"/>
-      <c r="P38" s="28"/>
-      <c r="Q38" s="28"/>
-      <c r="R38" s="28"/>
-      <c r="S38" s="28"/>
-      <c r="T38" s="28"/>
-      <c r="U38" s="28"/>
-      <c r="V38" s="28"/>
-      <c r="W38" s="28"/>
+      <c r="B38" s="21"/>
+      <c r="C38" s="21"/>
+      <c r="D38" s="21"/>
+      <c r="E38" s="21"/>
+      <c r="F38" s="21"/>
+      <c r="G38" s="21"/>
+      <c r="H38" s="21"/>
+      <c r="I38" s="21"/>
+      <c r="J38" s="21"/>
+      <c r="K38" s="21"/>
+      <c r="L38" s="21"/>
+      <c r="M38" s="21"/>
+      <c r="N38" s="21"/>
+      <c r="O38" s="21"/>
+      <c r="P38" s="21"/>
+      <c r="Q38" s="21"/>
+      <c r="R38" s="21"/>
+      <c r="S38" s="21"/>
+      <c r="T38" s="21"/>
+      <c r="U38" s="21"/>
+      <c r="V38" s="21"/>
+      <c r="W38" s="21"/>
     </row>
     <row r="39" spans="1:23" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="8" t="s">
@@ -1612,85 +1612,85 @@
       <c r="W39" s="8"/>
     </row>
     <row r="40" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A40" s="27" t="s">
+      <c r="A40" s="20" t="s">
+        <v>84</v>
+      </c>
+      <c r="B40" s="22"/>
+      <c r="C40" s="22"/>
+      <c r="D40" s="22"/>
+      <c r="E40" s="22"/>
+      <c r="F40" s="22"/>
+      <c r="G40" s="22"/>
+      <c r="H40" s="22"/>
+      <c r="I40" s="22"/>
+      <c r="J40" s="22"/>
+      <c r="K40" s="22"/>
+      <c r="L40" s="22"/>
+      <c r="M40" s="22"/>
+      <c r="N40" s="22"/>
+      <c r="O40" s="22"/>
+      <c r="P40" s="22"/>
+      <c r="Q40" s="22"/>
+      <c r="R40" s="22"/>
+      <c r="S40" s="22"/>
+      <c r="T40" s="22"/>
+      <c r="U40" s="22"/>
+      <c r="V40" s="22"/>
+      <c r="W40" s="22"/>
+    </row>
+    <row r="41" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A41" s="20" t="s">
         <v>85</v>
       </c>
-      <c r="B40" s="29"/>
-      <c r="C40" s="29"/>
-      <c r="D40" s="29"/>
-      <c r="E40" s="29"/>
-      <c r="F40" s="29"/>
-      <c r="G40" s="29"/>
-      <c r="H40" s="29"/>
-      <c r="I40" s="29"/>
-      <c r="J40" s="29"/>
-      <c r="K40" s="29"/>
-      <c r="L40" s="29"/>
-      <c r="M40" s="29"/>
-      <c r="N40" s="29"/>
-      <c r="O40" s="29"/>
-      <c r="P40" s="29"/>
-      <c r="Q40" s="29"/>
-      <c r="R40" s="29"/>
-      <c r="S40" s="29"/>
-      <c r="T40" s="29"/>
-      <c r="U40" s="29"/>
-      <c r="V40" s="29"/>
-      <c r="W40" s="29"/>
-    </row>
-    <row r="41" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A41" s="27" t="s">
+      <c r="B41" s="22"/>
+      <c r="C41" s="22"/>
+      <c r="D41" s="22"/>
+      <c r="E41" s="22"/>
+      <c r="F41" s="22"/>
+      <c r="G41" s="22"/>
+      <c r="H41" s="22"/>
+      <c r="I41" s="22"/>
+      <c r="J41" s="22"/>
+      <c r="K41" s="22"/>
+      <c r="L41" s="22"/>
+      <c r="M41" s="22"/>
+      <c r="N41" s="22"/>
+      <c r="O41" s="22"/>
+      <c r="P41" s="22"/>
+      <c r="Q41" s="22"/>
+      <c r="R41" s="22"/>
+      <c r="S41" s="22"/>
+      <c r="T41" s="22"/>
+      <c r="U41" s="22"/>
+      <c r="V41" s="22"/>
+      <c r="W41" s="22"/>
+    </row>
+    <row r="42" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A42" s="20" t="s">
         <v>86</v>
       </c>
-      <c r="B41" s="29"/>
-      <c r="C41" s="29"/>
-      <c r="D41" s="29"/>
-      <c r="E41" s="29"/>
-      <c r="F41" s="29"/>
-      <c r="G41" s="29"/>
-      <c r="H41" s="29"/>
-      <c r="I41" s="29"/>
-      <c r="J41" s="29"/>
-      <c r="K41" s="29"/>
-      <c r="L41" s="29"/>
-      <c r="M41" s="29"/>
-      <c r="N41" s="29"/>
-      <c r="O41" s="29"/>
-      <c r="P41" s="29"/>
-      <c r="Q41" s="29"/>
-      <c r="R41" s="29"/>
-      <c r="S41" s="29"/>
-      <c r="T41" s="29"/>
-      <c r="U41" s="29"/>
-      <c r="V41" s="29"/>
-      <c r="W41" s="29"/>
-    </row>
-    <row r="42" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A42" s="27" t="s">
-        <v>87</v>
-      </c>
-      <c r="B42" s="29"/>
-      <c r="C42" s="29"/>
-      <c r="D42" s="29"/>
-      <c r="E42" s="29"/>
-      <c r="F42" s="29"/>
-      <c r="G42" s="29"/>
-      <c r="H42" s="29"/>
-      <c r="I42" s="29"/>
-      <c r="J42" s="29"/>
-      <c r="K42" s="29"/>
-      <c r="L42" s="29"/>
-      <c r="M42" s="29"/>
-      <c r="N42" s="29"/>
-      <c r="O42" s="29"/>
-      <c r="P42" s="29"/>
-      <c r="Q42" s="29"/>
-      <c r="R42" s="29"/>
-      <c r="S42" s="29"/>
-      <c r="T42" s="29"/>
-      <c r="U42" s="29"/>
-      <c r="V42" s="29"/>
-      <c r="W42" s="29"/>
+      <c r="B42" s="22"/>
+      <c r="C42" s="22"/>
+      <c r="D42" s="22"/>
+      <c r="E42" s="22"/>
+      <c r="F42" s="22"/>
+      <c r="G42" s="22"/>
+      <c r="H42" s="22"/>
+      <c r="I42" s="22"/>
+      <c r="J42" s="22"/>
+      <c r="K42" s="22"/>
+      <c r="L42" s="22"/>
+      <c r="M42" s="22"/>
+      <c r="N42" s="22"/>
+      <c r="O42" s="22"/>
+      <c r="P42" s="22"/>
+      <c r="Q42" s="22"/>
+      <c r="R42" s="22"/>
+      <c r="S42" s="22"/>
+      <c r="T42" s="22"/>
+      <c r="U42" s="22"/>
+      <c r="V42" s="22"/>
+      <c r="W42" s="22"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -1736,24 +1736,24 @@
       </c>
     </row>
     <row r="8" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="21" t="s">
+      <c r="B8" s="27" t="s">
         <v>30</v>
       </c>
-      <c r="C8" s="21"/>
-      <c r="D8" s="21"/>
-      <c r="E8" s="21"/>
-      <c r="F8" s="21"/>
-      <c r="G8" s="21"/>
-      <c r="H8" s="21"/>
-      <c r="I8" s="21"/>
-      <c r="J8" s="21"/>
-      <c r="K8" s="22" t="s">
+      <c r="C8" s="27"/>
+      <c r="D8" s="27"/>
+      <c r="E8" s="27"/>
+      <c r="F8" s="27"/>
+      <c r="G8" s="27"/>
+      <c r="H8" s="27"/>
+      <c r="I8" s="27"/>
+      <c r="J8" s="27"/>
+      <c r="K8" s="28" t="s">
         <v>31</v>
       </c>
-      <c r="L8" s="23" t="s">
+      <c r="L8" s="29" t="s">
         <v>32</v>
       </c>
-      <c r="M8" s="23" t="s">
+      <c r="M8" s="29" t="s">
         <v>33</v>
       </c>
       <c r="N8" s="13"/>
@@ -1786,9 +1786,9 @@
       <c r="J9" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="K9" s="22"/>
-      <c r="L9" s="23"/>
-      <c r="M9" s="23"/>
+      <c r="K9" s="28"/>
+      <c r="L9" s="29"/>
+      <c r="M9" s="29"/>
       <c r="N9" s="13"/>
     </row>
     <row r="10" spans="2:16" ht="15.75" x14ac:dyDescent="0.25">
@@ -1855,7 +1855,7 @@
         <v>1296</v>
       </c>
       <c r="P12" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="13" spans="2:16" x14ac:dyDescent="0.25">
@@ -1876,7 +1876,7 @@
       </c>
       <c r="M13" s="15"/>
       <c r="P13" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="14" spans="2:16" x14ac:dyDescent="0.25">

</xml_diff>